<commit_message>
docs: add API filter test cases (TC-API-011, TC-API-012)
</commit_message>
<xml_diff>
--- a/docs/05_api_requirements.xlsx
+++ b/docs/05_api_requirements.xlsx
@@ -498,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -805,6 +805,60 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>REQ-API-011</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>GET /booking</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>İsim (firstname/lastname) query parametreleriyle rezervasyonlar filtrelenebilmelidir (200 + eşleşen id listesi).</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>REQ-API-012</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>GET /booking</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Tarih (checkin/checkout) query parametreleriyle rezervasyonlar filtrelenebilmelidir (200 + eşleşen id listesi).</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>